<commit_message>
ajuste na base de dados
</commit_message>
<xml_diff>
--- a/dados/nomes_usuais.xlsx
+++ b/dados/nomes_usuais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amaggicombr-my.sharepoint.com/personal/hiago_andre_amaggi_com_br/Documents/Área de Trabalho/catalogoPecas/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E773DA3B-55AF-49D2-93F9-A3811158B3A4}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_AD4D361C20488DEA4E38A03414D973025ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F4B1027-81F3-421D-8E75-5DEFB80CE880}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4155" yWindow="4155" windowWidth="15900" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="12150" windowHeight="20745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -489,12 +489,6 @@
     <t>KIT TAPA PO RANDON (PAR DE ESPELHO)</t>
   </si>
   <si>
-    <t>KIT TAPA PO FACCHINI LE (PAR DE ESPELHO)</t>
-  </si>
-  <si>
-    <t>KIT TAPA PO FACCHINI LD (PAR DE ESPELHO)</t>
-  </si>
-  <si>
     <t>LOCTITTE (TRAVA PARAFUSO)</t>
   </si>
   <si>
@@ -1315,6 +1309,12 @@
   </si>
   <si>
     <t>material</t>
+  </si>
+  <si>
+    <t>KIT TAPA PO FACCHINI LE (ESPELHO)</t>
+  </si>
+  <si>
+    <t>KIT TAPA PO FACCHINI LD (ESPELHO)</t>
   </si>
 </sst>
 </file>
@@ -1553,6 +1553,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1827,10 +1831,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -2422,7 +2426,7 @@
         <v>341430</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3078,7 +3082,7 @@
         <v>1040097070</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>154</v>
+        <v>428</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3086,7 +3090,7 @@
         <v>1040097068</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>155</v>
+        <v>429</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3094,7 +3098,7 @@
         <v>22004</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3102,7 +3106,7 @@
         <v>1010058554</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3110,7 +3114,7 @@
         <v>1010027308</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3118,7 +3122,7 @@
         <v>1040077383</v>
       </c>
       <c r="B162" s="6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3126,7 +3130,7 @@
         <v>1010025482</v>
       </c>
       <c r="B163" s="6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="164" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3134,7 +3138,7 @@
         <v>1010025509</v>
       </c>
       <c r="B164" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3142,7 +3146,7 @@
         <v>1010027789</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="166" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3150,7 +3154,7 @@
         <v>1010027790</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3158,7 +3162,7 @@
         <v>1010018301</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3166,7 +3170,7 @@
         <v>1010031616</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3174,7 +3178,7 @@
         <v>1010053728</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3182,7 +3186,7 @@
         <v>1010020758</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3190,7 +3194,7 @@
         <v>1010020781</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="172" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3198,7 +3202,7 @@
         <v>1010058426</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3206,7 +3210,7 @@
         <v>1010059332</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="174" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3214,7 +3218,7 @@
         <v>1040077389</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3222,7 +3226,7 @@
         <v>1010021364</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3230,7 +3234,7 @@
         <v>1010021541</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3238,7 +3242,7 @@
         <v>1010021955</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3246,7 +3250,7 @@
         <v>1040077388</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3254,7 +3258,7 @@
         <v>1010058100</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3262,7 +3266,7 @@
         <v>1010020524</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="181" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3270,7 +3274,7 @@
         <v>1010021958</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="182" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3278,7 +3282,7 @@
         <v>1010019756</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="183" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3286,7 +3290,7 @@
         <v>1010019752</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="184" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3294,7 +3298,7 @@
         <v>409639</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="185" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3302,7 +3306,7 @@
         <v>1010047089</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="186" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3310,7 +3314,7 @@
         <v>1040084107</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3318,7 +3322,7 @@
         <v>405588</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="188" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3326,7 +3330,7 @@
         <v>424298</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="189" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3334,7 +3338,7 @@
         <v>421847</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="190" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3342,7 +3346,7 @@
         <v>431573</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="191" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3350,7 +3354,7 @@
         <v>1010021581</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="192" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3358,7 +3362,7 @@
         <v>412413</v>
       </c>
       <c r="B192" s="14" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="193" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3366,7 +3370,7 @@
         <v>1010022606</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3374,7 +3378,7 @@
         <v>1010003527</v>
       </c>
       <c r="B194" s="14" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3382,7 +3386,7 @@
         <v>422027</v>
       </c>
       <c r="B195" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="196" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3390,7 +3394,7 @@
         <v>1010011313</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3398,7 +3402,7 @@
         <v>27051</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="198" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3406,7 +3410,7 @@
         <v>1010011304</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="199" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3414,7 +3418,7 @@
         <v>35659</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="200" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3422,7 +3426,7 @@
         <v>1040077390</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="201" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3430,7 +3434,7 @@
         <v>1010021542</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="202" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3438,7 +3442,7 @@
         <v>1010021733</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="203" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3446,7 +3450,7 @@
         <v>1010011379</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="204" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3454,7 +3458,7 @@
         <v>1010003279</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="205" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3462,7 +3466,7 @@
         <v>1010011380</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3470,7 +3474,7 @@
         <v>351197</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="207" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3478,7 +3482,7 @@
         <v>1010011286</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="208" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3486,7 +3490,7 @@
         <v>2479</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="209" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3494,7 +3498,7 @@
         <v>1010011382</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="210" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3502,7 +3506,7 @@
         <v>1010055703</v>
       </c>
       <c r="B210" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="211" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3510,7 +3514,7 @@
         <v>4165</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="212" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3518,7 +3522,7 @@
         <v>301626</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="213" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3526,7 +3530,7 @@
         <v>429495</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="214" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3534,7 +3538,7 @@
         <v>162998</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="215" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3542,7 +3546,7 @@
         <v>432657</v>
       </c>
       <c r="B215" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="216" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3550,7 +3554,7 @@
         <v>1010021929</v>
       </c>
       <c r="B216" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="217" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3558,7 +3562,7 @@
         <v>428065</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3566,7 +3570,7 @@
         <v>1010003404</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="219" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3574,7 +3578,7 @@
         <v>1010003322</v>
       </c>
       <c r="B219" s="14" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="220" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3582,7 +3586,7 @@
         <v>17738</v>
       </c>
       <c r="B220" s="14" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="221" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3590,7 +3594,7 @@
         <v>270373</v>
       </c>
       <c r="B221" s="14" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3598,7 +3602,7 @@
         <v>1040077391</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="223" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3606,7 +3610,7 @@
         <v>1010058624</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3614,7 +3618,7 @@
         <v>1010024661</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="225" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3622,7 +3626,7 @@
         <v>1040019315</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="226" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3630,7 +3634,7 @@
         <v>1010021089</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="227" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3638,7 +3642,7 @@
         <v>1040017264</v>
       </c>
       <c r="B227" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="228" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3646,7 +3650,7 @@
         <v>1010051765</v>
       </c>
       <c r="B228" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="229" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3654,7 +3658,7 @@
         <v>1010035272</v>
       </c>
       <c r="B229" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="230" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3662,7 +3666,7 @@
         <v>1040077392</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="231" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3670,7 +3674,7 @@
         <v>1040077393</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="232" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3678,7 +3682,7 @@
         <v>1040077395</v>
       </c>
       <c r="B232" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="233" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3686,7 +3690,7 @@
         <v>1040077401</v>
       </c>
       <c r="B233" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="234" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3694,7 +3698,7 @@
         <v>27572</v>
       </c>
       <c r="B234" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="235" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3702,7 +3706,7 @@
         <v>18745</v>
       </c>
       <c r="B235" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="236" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3710,7 +3714,7 @@
         <v>1040077396</v>
       </c>
       <c r="B236" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="237" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3718,7 +3722,7 @@
         <v>1010036546</v>
       </c>
       <c r="B237" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="238" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3726,7 +3730,7 @@
         <v>1010014049</v>
       </c>
       <c r="B238" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="239" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3734,7 +3738,7 @@
         <v>1010025148</v>
       </c>
       <c r="B239" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="240" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3742,7 +3746,7 @@
         <v>1040077394</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3750,7 +3754,7 @@
         <v>1040077400</v>
       </c>
       <c r="B241" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="242" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3758,7 +3762,7 @@
         <v>1040079329</v>
       </c>
       <c r="B242" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="243" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3766,7 +3770,7 @@
         <v>1040040957</v>
       </c>
       <c r="B243" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3774,7 +3778,7 @@
         <v>1040077398</v>
       </c>
       <c r="B244" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="245" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3782,7 +3786,7 @@
         <v>1010031545</v>
       </c>
       <c r="B245" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="246" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3790,7 +3794,7 @@
         <v>1010053128</v>
       </c>
       <c r="B246" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="247" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3798,7 +3802,7 @@
         <v>1010010599</v>
       </c>
       <c r="B247" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="248" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3806,7 +3810,7 @@
         <v>1010056064</v>
       </c>
       <c r="B248" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3814,7 +3818,7 @@
         <v>5389</v>
       </c>
       <c r="B249" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3822,7 +3826,7 @@
         <v>264250</v>
       </c>
       <c r="B250" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3830,7 +3834,7 @@
         <v>1010055970</v>
       </c>
       <c r="B251" s="4" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3838,7 +3842,7 @@
         <v>181395</v>
       </c>
       <c r="B252" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="253" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3846,7 +3850,7 @@
         <v>1010055962</v>
       </c>
       <c r="B253" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="254" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3854,7 +3858,7 @@
         <v>1010003578</v>
       </c>
       <c r="B254" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="255" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3862,7 +3866,7 @@
         <v>332891</v>
       </c>
       <c r="B255" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="256" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3870,7 +3874,7 @@
         <v>17727</v>
       </c>
       <c r="B256" s="4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="257" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3878,7 +3882,7 @@
         <v>17918</v>
       </c>
       <c r="B257" s="4" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="258" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3886,7 +3890,7 @@
         <v>1010020554</v>
       </c>
       <c r="B258" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="259" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3894,7 +3898,7 @@
         <v>1040085949</v>
       </c>
       <c r="B259" s="4" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="260" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3902,7 +3906,7 @@
         <v>1010062938</v>
       </c>
       <c r="B260" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="261" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3910,7 +3914,7 @@
         <v>1010062086</v>
       </c>
       <c r="B261" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="262" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3918,7 +3922,7 @@
         <v>1010062087</v>
       </c>
       <c r="B262" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="263" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3926,7 +3930,7 @@
         <v>1040077373</v>
       </c>
       <c r="B263" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="264" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3934,7 +3938,7 @@
         <v>1040077372</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="265" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3942,7 +3946,7 @@
         <v>1040097154</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="266" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3950,7 +3954,7 @@
         <v>1010042579</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="267" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3958,7 +3962,7 @@
         <v>1010029427</v>
       </c>
       <c r="B267" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="268" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3966,7 +3970,7 @@
         <v>133108</v>
       </c>
       <c r="B268" s="4" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="269" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3974,7 +3978,7 @@
         <v>269427</v>
       </c>
       <c r="B269" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="270" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3982,7 +3986,7 @@
         <v>298227</v>
       </c>
       <c r="B270" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="271" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3990,7 +3994,7 @@
         <v>1010062285</v>
       </c>
       <c r="B271" s="4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="272" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -3998,7 +4002,7 @@
         <v>1010058052</v>
       </c>
       <c r="B272" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="273" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4006,7 +4010,7 @@
         <v>1010050033</v>
       </c>
       <c r="B273" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="274" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4014,7 +4018,7 @@
         <v>1040098869</v>
       </c>
       <c r="B274" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="275" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4022,7 +4026,7 @@
         <v>1010056523</v>
       </c>
       <c r="B275" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="276" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4030,7 +4034,7 @@
         <v>1010062045</v>
       </c>
       <c r="B276" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="277" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4038,7 +4042,7 @@
         <v>1040097575</v>
       </c>
       <c r="B277" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="278" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4046,7 +4050,7 @@
         <v>1040098437</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="279" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4054,7 +4058,7 @@
         <v>1010040346</v>
       </c>
       <c r="B279" s="4" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="280" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4062,7 +4066,7 @@
         <v>1010021543</v>
       </c>
       <c r="B280" s="4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="281" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4070,7 +4074,7 @@
         <v>1040077397</v>
       </c>
       <c r="B281" s="4" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="282" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4078,7 +4082,7 @@
         <v>1040094213</v>
       </c>
       <c r="B282" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="283" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4086,7 +4090,7 @@
         <v>406060</v>
       </c>
       <c r="B283" s="4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="284" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4094,7 +4098,7 @@
         <v>1010042564</v>
       </c>
       <c r="B284" s="4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="285" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4102,7 +4106,7 @@
         <v>1010042688</v>
       </c>
       <c r="B285" s="4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="286" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4110,7 +4114,7 @@
         <v>1010040133</v>
       </c>
       <c r="B286" s="4" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="287" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4118,7 +4122,7 @@
         <v>1010039879</v>
       </c>
       <c r="B287" s="4" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="288" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4126,7 +4130,7 @@
         <v>62608</v>
       </c>
       <c r="B288" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="289" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4134,7 +4138,7 @@
         <v>1040098603</v>
       </c>
       <c r="B289" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="290" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4142,7 +4146,7 @@
         <v>1040017266</v>
       </c>
       <c r="B290" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="291" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4150,7 +4154,7 @@
         <v>1010063326</v>
       </c>
       <c r="B291" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="292" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4158,7 +4162,7 @@
         <v>1010050574</v>
       </c>
       <c r="B292" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="293" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4166,7 +4170,7 @@
         <v>1040087856</v>
       </c>
       <c r="B293" s="4" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="294" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4174,7 +4178,7 @@
         <v>1040019838</v>
       </c>
       <c r="B294" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="295" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4182,7 +4186,7 @@
         <v>1010042882</v>
       </c>
       <c r="B295" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="296" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4190,7 +4194,7 @@
         <v>1010042873</v>
       </c>
       <c r="B296" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="297" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4198,7 +4202,7 @@
         <v>1010059549</v>
       </c>
       <c r="B297" s="4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="298" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4206,7 +4210,7 @@
         <v>1010020552</v>
       </c>
       <c r="B298" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="299" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4214,7 +4218,7 @@
         <v>1040078895</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="300" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4222,7 +4226,7 @@
         <v>1040024309</v>
       </c>
       <c r="B300" s="4" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="301" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4230,7 +4234,7 @@
         <v>1040024323</v>
       </c>
       <c r="B301" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="302" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4238,7 +4242,7 @@
         <v>1040024322</v>
       </c>
       <c r="B302" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="303" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4246,7 +4250,7 @@
         <v>417694</v>
       </c>
       <c r="B303" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="304" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4254,7 +4258,7 @@
         <v>1010059685</v>
       </c>
       <c r="B304" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="305" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4262,7 +4266,7 @@
         <v>1010059687</v>
       </c>
       <c r="B305" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="306" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4270,7 +4274,7 @@
         <v>1010077469</v>
       </c>
       <c r="B306" s="4" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="307" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4278,15 +4282,15 @@
         <v>1010077470</v>
       </c>
       <c r="B307" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="308" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A308" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B308" s="14" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="309" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4294,7 +4298,7 @@
         <v>1010084108</v>
       </c>
       <c r="B309" s="4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="310" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4302,7 +4306,7 @@
         <v>1040043537</v>
       </c>
       <c r="B310" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="311" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4310,7 +4314,7 @@
         <v>1010046401</v>
       </c>
       <c r="B311" s="4" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="312" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4318,7 +4322,7 @@
         <v>1010062007</v>
       </c>
       <c r="B312" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="313" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4326,7 +4330,7 @@
         <v>1010051284</v>
       </c>
       <c r="B313" s="4" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="314" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4334,7 +4338,7 @@
         <v>1010027788</v>
       </c>
       <c r="B314" s="4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="315" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4342,7 +4346,7 @@
         <v>1010027786</v>
       </c>
       <c r="B315" s="4" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="316" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4350,7 +4354,7 @@
         <v>1010026889</v>
       </c>
       <c r="B316" s="4" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="317" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4358,7 +4362,7 @@
         <v>1010042358</v>
       </c>
       <c r="B317" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="318" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4366,7 +4370,7 @@
         <v>1040023848</v>
       </c>
       <c r="B318" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="319" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4374,7 +4378,7 @@
         <v>1010042341</v>
       </c>
       <c r="B319" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="320" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4382,7 +4386,7 @@
         <v>1040023858</v>
       </c>
       <c r="B320" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="321" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4390,7 +4394,7 @@
         <v>1040023843</v>
       </c>
       <c r="B321" s="4" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="322" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4398,7 +4402,7 @@
         <v>1040077411</v>
       </c>
       <c r="B322" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="323" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4406,7 +4410,7 @@
         <v>1040077410</v>
       </c>
       <c r="B323" s="4" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="324" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4414,7 +4418,7 @@
         <v>1010062008</v>
       </c>
       <c r="B324" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="325" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4422,7 +4426,7 @@
         <v>1040040960</v>
       </c>
       <c r="B325" s="4" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="326" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4430,7 +4434,7 @@
         <v>409578</v>
       </c>
       <c r="B326" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="327" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4438,7 +4442,7 @@
         <v>1040077360</v>
       </c>
       <c r="B327" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="328" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4446,7 +4450,7 @@
         <v>1010064470</v>
       </c>
       <c r="B328" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="329" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4454,7 +4458,7 @@
         <v>1010021991</v>
       </c>
       <c r="B329" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="330" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4462,7 +4466,7 @@
         <v>1010021960</v>
       </c>
       <c r="B330" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="331" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4470,7 +4474,7 @@
         <v>1010031545</v>
       </c>
       <c r="B331" s="4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="332" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4478,7 +4482,7 @@
         <v>1010022590</v>
       </c>
       <c r="B332" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="333" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4486,13 +4490,13 @@
         <v>1040098643</v>
       </c>
       <c r="B333" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="334" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A334" s="4"/>
       <c r="B334" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="335" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4500,7 +4504,7 @@
         <v>1010046550</v>
       </c>
       <c r="B335" s="4" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="336" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4508,7 +4512,7 @@
         <v>1010046402</v>
       </c>
       <c r="B336" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="337" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4516,7 +4520,7 @@
         <v>1010060291</v>
       </c>
       <c r="B337" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="338" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4524,7 +4528,7 @@
         <v>1010050920</v>
       </c>
       <c r="B338" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="339" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4532,7 +4536,7 @@
         <v>1040077412</v>
       </c>
       <c r="B339" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="340" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4540,7 +4544,7 @@
         <v>1010042609</v>
       </c>
       <c r="B340" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="341" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4548,7 +4552,7 @@
         <v>417701</v>
       </c>
       <c r="B341" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="342" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4556,7 +4560,7 @@
         <v>399384</v>
       </c>
       <c r="B342" s="4" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="343" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4564,7 +4568,7 @@
         <v>1040077345</v>
       </c>
       <c r="B343" s="4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="344" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4572,7 +4576,7 @@
         <v>297290</v>
       </c>
       <c r="B344" s="4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="345" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4580,7 +4584,7 @@
         <v>399253</v>
       </c>
       <c r="B345" s="4" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="346" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4588,7 +4592,7 @@
         <v>377363</v>
       </c>
       <c r="B346" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="347" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4596,7 +4600,7 @@
         <v>405556</v>
       </c>
       <c r="B347" s="4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="348" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4604,7 +4608,7 @@
         <v>405590</v>
       </c>
       <c r="B348" s="4" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="349" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4612,7 +4616,7 @@
         <v>405591</v>
       </c>
       <c r="B349" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="350" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4620,7 +4624,7 @@
         <v>1010003966</v>
       </c>
       <c r="B350" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="351" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4628,7 +4632,7 @@
         <v>1010003967</v>
       </c>
       <c r="B351" s="4" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="352" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4636,7 +4640,7 @@
         <v>65219</v>
       </c>
       <c r="B352" s="4" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="353" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4644,7 +4648,7 @@
         <v>10168</v>
       </c>
       <c r="B353" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="354" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4652,7 +4656,7 @@
         <v>180778</v>
       </c>
       <c r="B354" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="355" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4660,7 +4664,7 @@
         <v>1040077414</v>
       </c>
       <c r="B355" s="4" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="356" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4668,7 +4672,7 @@
         <v>1010018482</v>
       </c>
       <c r="B356" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="357" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4676,7 +4680,7 @@
         <v>409903</v>
       </c>
       <c r="B357" s="4" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="358" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4684,7 +4688,7 @@
         <v>418427</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="359" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4692,7 +4696,7 @@
         <v>1010027285</v>
       </c>
       <c r="B359" s="4" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="360" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4700,7 +4704,7 @@
         <v>1040077413</v>
       </c>
       <c r="B360" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="361" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4708,7 +4712,7 @@
         <v>416554</v>
       </c>
       <c r="B361" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="362" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4716,7 +4720,7 @@
         <v>1010022819</v>
       </c>
       <c r="B362" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="363" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4724,7 +4728,7 @@
         <v>1010052853</v>
       </c>
       <c r="B363" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="364" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4732,7 +4736,7 @@
         <v>433362</v>
       </c>
       <c r="B364" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="365" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4740,7 +4744,7 @@
         <v>1010008578</v>
       </c>
       <c r="B365" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="366" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4748,7 +4752,7 @@
         <v>1010031694</v>
       </c>
       <c r="B366" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="367" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4756,7 +4760,7 @@
         <v>1010051997</v>
       </c>
       <c r="B367" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="368" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4764,7 +4768,7 @@
         <v>1010022601</v>
       </c>
       <c r="B368" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="369" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4772,7 +4776,7 @@
         <v>1010054278</v>
       </c>
       <c r="B369" s="4" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="370" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4780,7 +4784,7 @@
         <v>1010083462</v>
       </c>
       <c r="B370" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="371" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4788,7 +4792,7 @@
         <v>1010027772</v>
       </c>
       <c r="B371" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="372" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4796,7 +4800,7 @@
         <v>300186</v>
       </c>
       <c r="B372" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="373" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4804,7 +4808,7 @@
         <v>214055</v>
       </c>
       <c r="B373" s="14" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="374" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4812,7 +4816,7 @@
         <v>1010021956</v>
       </c>
       <c r="B374" s="14" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="375" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4820,7 +4824,7 @@
         <v>1010026464</v>
       </c>
       <c r="B375" s="14" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="376" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4828,7 +4832,7 @@
         <v>1010021957</v>
       </c>
       <c r="B376" s="4" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="377" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4836,7 +4840,7 @@
         <v>1010026462</v>
       </c>
       <c r="B377" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="378" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4844,7 +4848,7 @@
         <v>1010026551</v>
       </c>
       <c r="B378" s="4" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="379" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4852,7 +4856,7 @@
         <v>1010042554</v>
       </c>
       <c r="B379" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="380" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4860,7 +4864,7 @@
         <v>1010039904</v>
       </c>
       <c r="B380" s="4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="381" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4868,7 +4872,7 @@
         <v>1010060205</v>
       </c>
       <c r="B381" s="4" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="382" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4876,7 +4880,7 @@
         <v>1010060206</v>
       </c>
       <c r="B382" s="4" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="383" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4884,7 +4888,7 @@
         <v>1010077431</v>
       </c>
       <c r="B383" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="384" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4892,7 +4896,7 @@
         <v>1010077503</v>
       </c>
       <c r="B384" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="385" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4900,7 +4904,7 @@
         <v>386009</v>
       </c>
       <c r="B385" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="386" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4908,7 +4912,7 @@
         <v>1010080958</v>
       </c>
       <c r="B386" s="4" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="387" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4916,7 +4920,7 @@
         <v>20191</v>
       </c>
       <c r="B387" s="4" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="388" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4924,7 +4928,7 @@
         <v>431445</v>
       </c>
       <c r="B388" s="4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="389" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4932,7 +4936,7 @@
         <v>431463</v>
       </c>
       <c r="B389" s="4" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="390" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4940,7 +4944,7 @@
         <v>431464</v>
       </c>
       <c r="B390" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="391" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4948,7 +4952,7 @@
         <v>1010024158</v>
       </c>
       <c r="B391" s="6" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="392" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4956,7 +4960,7 @@
         <v>1010024131</v>
       </c>
       <c r="B392" s="6" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="393" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4964,7 +4968,7 @@
         <v>1010007160</v>
       </c>
       <c r="B393" s="4" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="394" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4972,7 +4976,7 @@
         <v>1010023642</v>
       </c>
       <c r="B394" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="395" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4980,7 +4984,7 @@
         <v>1010007193</v>
       </c>
       <c r="B395" s="5" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="396" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4988,7 +4992,7 @@
         <v>1010042637</v>
       </c>
       <c r="B396" s="4" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="397" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -4996,7 +5000,7 @@
         <v>1040075323</v>
       </c>
       <c r="B397" s="4" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="398" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5004,7 +5008,7 @@
         <v>1040075324</v>
       </c>
       <c r="B398" s="6" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="399" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5012,7 +5016,7 @@
         <v>1040083312</v>
       </c>
       <c r="B399" s="6" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="400" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5020,7 +5024,7 @@
         <v>1040077661</v>
       </c>
       <c r="B400" s="6" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="401" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5028,7 +5032,7 @@
         <v>409638</v>
       </c>
       <c r="B401" s="19" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="402" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5036,7 +5040,7 @@
         <v>1040017489</v>
       </c>
       <c r="B402" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="403" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5044,7 +5048,7 @@
         <v>400174</v>
       </c>
       <c r="B403" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="404" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5052,7 +5056,7 @@
         <v>400175</v>
       </c>
       <c r="B404" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="405" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5060,7 +5064,7 @@
         <v>1040017505</v>
       </c>
       <c r="B405" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="406" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5068,7 +5072,7 @@
         <v>1040017503</v>
       </c>
       <c r="B406" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="407" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5076,7 +5080,7 @@
         <v>1010046445</v>
       </c>
       <c r="B407" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="408" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5084,7 +5088,7 @@
         <v>1010021033</v>
       </c>
       <c r="B408" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="409" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5092,7 +5096,7 @@
         <v>24950</v>
       </c>
       <c r="B409" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="410" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5100,7 +5104,7 @@
         <v>1010016356</v>
       </c>
       <c r="B410" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="411" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5108,7 +5112,7 @@
         <v>400228</v>
       </c>
       <c r="B411" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="412" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5116,7 +5120,7 @@
         <v>1010052021</v>
       </c>
       <c r="B412" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="413" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5124,7 +5128,7 @@
         <v>1040091721</v>
       </c>
       <c r="B413" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="414" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5132,7 +5136,7 @@
         <v>1010062022</v>
       </c>
       <c r="B414" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="415" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5140,7 +5144,7 @@
         <v>18336</v>
       </c>
       <c r="B415" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="416" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5148,7 +5152,7 @@
         <v>229205</v>
       </c>
       <c r="B416" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="417" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5156,7 +5160,7 @@
         <v>60671</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="418" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5164,7 +5168,7 @@
         <v>1010059726</v>
       </c>
       <c r="B418" s="4" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="419" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5172,7 +5176,7 @@
         <v>1010008144</v>
       </c>
       <c r="B419" s="4" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="420" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5180,7 +5184,7 @@
         <v>1010007244</v>
       </c>
       <c r="B420" s="4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="421" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5188,7 +5192,7 @@
         <v>1010006827</v>
       </c>
       <c r="B421" s="4" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="422" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5196,7 +5200,7 @@
         <v>1040075426</v>
       </c>
       <c r="B422" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="423" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5204,7 +5208,7 @@
         <v>1040075427</v>
       </c>
       <c r="B423" s="4" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="424" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5212,7 +5216,7 @@
         <v>401167</v>
       </c>
       <c r="B424" s="4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="425" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5220,7 +5224,7 @@
         <v>403459</v>
       </c>
       <c r="B425" s="4" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="426" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5228,7 +5232,7 @@
         <v>300296</v>
       </c>
       <c r="B426" s="4" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="427" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5236,7 +5240,7 @@
         <v>1010026973</v>
       </c>
       <c r="B427" s="4" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="428" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -5244,7 +5248,7 @@
         <v>1040017204</v>
       </c>
       <c r="B428" s="4" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="429" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>